<commit_message>
Contextualisation Sénégal : références Maman Tontine et MaTontine
- docs/00 : comparatif, reprises, différenciation, enjeu du prix de retrait, CI vs Sénégal
- Coffres de groupe (associations, dahiras, GIE…) : catégories, adhésion par code,
  suivi des cotisations payé / partiel / impayé par période
- Rappels automatiques J-1 / J0 (cotisations de tontine et échéances de crédit)
- Invitation par QR code, WhatsApp et lien smartfin://rejoindre/…
- Modèle financier : levier « pots retirés sans frais » pour chiffrer l'alignement tarifaire

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DBrAbxmxcXp2zsbgbJRBkp
</commit_message>
<xml_diff>
--- a/finance/SMARTFIN_modele_financier.xlsx
+++ b/finance/SMARTFIN_modele_financier.xlsx
@@ -29,7 +29,7 @@
     <author>Unknown Author</author>
   </authors>
   <commentList>
-    <comment ref="C45" authorId="0">
+    <comment ref="C46" authorId="0">
       <text>
         <r>
           <rPr>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="375" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="231">
   <si>
     <t xml:space="preserve">SMARTFIN — Synthèse financière</t>
   </si>
@@ -207,7 +207,13 @@
     <t xml:space="preserve">Commission SMARTFIN sur chaque pot versé</t>
   </si>
   <si>
-    <t xml:space="preserve">backend/src/pricing.ts → tontine.commissionRate</t>
+    <t xml:space="preserve">backend/src/pricing.ts → tontine.commissionRate. Référence marché : Maman Tontine (Sénégal) affiche 1 % de frais de plateforme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Part des pots retirés vers Mobile Money SANS frais de retrait</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Levier concurrentiel : chez Maman Tontine, le tour est reçu directement sur Wave / Orange Money pour 1 % au total. 0 % = tarif actuel (retrait 1,5 %).</t>
   </si>
   <si>
     <t xml:space="preserve">Microfinance (crédit financé par le SFD partenaire)</t>
@@ -559,6 +565,9 @@
   </si>
   <si>
     <t xml:space="preserve">dont retraits payants</t>
+  </si>
+  <si>
+    <t xml:space="preserve">retraits − offerts SMARTFIN+ − pots retirés sans frais (levier concurrentiel)</t>
   </si>
   <si>
     <t xml:space="preserve">Encours moyen clients (float)</t>
@@ -1835,7 +1844,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H64"/>
+  <dimension ref="A1:H65"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
@@ -2061,64 +2070,52 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="11" t="s">
+      <c r="A14" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="B14" s="12"/>
-      <c r="C14" s="12"/>
-      <c r="D14" s="12"/>
-      <c r="E14" s="12"/>
-      <c r="F14" s="12"/>
-      <c r="G14" s="12"/>
-      <c r="H14" s="12"/>
+      <c r="B14" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C14" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="15" t="s">
+        <v>55</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C15" s="19" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="D15" s="19" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="E15" s="19" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="F15" s="19" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="G15" s="19" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="H15" s="15" t="s">
+      <c r="A15" s="11" t="s">
         <v>56</v>
       </c>
+      <c r="B15" s="12"/>
+      <c r="C15" s="12"/>
+      <c r="D15" s="12"/>
+      <c r="E15" s="12"/>
+      <c r="F15" s="12"/>
+      <c r="G15" s="12"/>
+      <c r="H15" s="12"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
         <v>57</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="C16" s="20" t="n">
-        <v>40000</v>
-      </c>
-      <c r="D16" s="20" t="n">
-        <v>45000</v>
-      </c>
-      <c r="E16" s="20" t="n">
-        <v>50000</v>
-      </c>
-      <c r="F16" s="20" t="n">
-        <v>55000</v>
-      </c>
-      <c r="G16" s="20" t="n">
-        <v>60000</v>
+        <v>20</v>
+      </c>
+      <c r="C16" s="19" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D16" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E16" s="19" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F16" s="19" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G16" s="19" t="n">
+        <v>0.2</v>
       </c>
       <c r="H16" s="15" t="s">
         <v>58</v>
@@ -2129,26 +2126,38 @@
         <v>59</v>
       </c>
       <c r="B17" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C17" s="20" t="n">
+        <v>40000</v>
+      </c>
+      <c r="D17" s="20" t="n">
+        <v>45000</v>
+      </c>
+      <c r="E17" s="20" t="n">
+        <v>50000</v>
+      </c>
+      <c r="F17" s="20" t="n">
+        <v>55000</v>
+      </c>
+      <c r="G17" s="20" t="n">
+        <v>60000</v>
+      </c>
+      <c r="H17" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="C17" s="20" t="n">
-        <v>2</v>
-      </c>
-      <c r="H17" s="15"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
         <v>61</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C18" s="21" t="n">
-        <v>0.015</v>
-      </c>
-      <c r="H18" s="15" t="s">
         <v>62</v>
       </c>
+      <c r="C18" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="H18" s="15"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
@@ -2157,20 +2166,8 @@
       <c r="B19" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C19" s="19" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="D19" s="19" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="E19" s="19" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="F19" s="19" t="n">
-        <v>0.07</v>
-      </c>
-      <c r="G19" s="19" t="n">
-        <v>0.08</v>
+      <c r="C19" s="21" t="n">
+        <v>0.015</v>
       </c>
       <c r="H19" s="15" t="s">
         <v>64</v>
@@ -2181,36 +2178,36 @@
         <v>65</v>
       </c>
       <c r="B20" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C20" s="19" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D20" s="19" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="E20" s="19" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F20" s="19" t="n">
+        <v>0.07</v>
+      </c>
+      <c r="G20" s="19" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="H20" s="15" t="s">
         <v>66</v>
-      </c>
-      <c r="C20" s="20" t="n">
-        <v>2</v>
-      </c>
-      <c r="H20" s="15" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B21" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="B21" s="6" t="s">
-        <v>25</v>
-      </c>
       <c r="C21" s="20" t="n">
-        <v>75000</v>
-      </c>
-      <c r="D21" s="20" t="n">
-        <v>90000</v>
-      </c>
-      <c r="E21" s="20" t="n">
-        <v>100000</v>
-      </c>
-      <c r="F21" s="20" t="n">
-        <v>120000</v>
-      </c>
-      <c r="G21" s="20" t="n">
-        <v>140000</v>
+        <v>2</v>
       </c>
       <c r="H21" s="15" t="s">
         <v>69</v>
@@ -2221,38 +2218,50 @@
         <v>70</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>60</v>
+        <v>25</v>
       </c>
       <c r="C22" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="H22" s="15"/>
+        <v>75000</v>
+      </c>
+      <c r="D22" s="20" t="n">
+        <v>90000</v>
+      </c>
+      <c r="E22" s="20" t="n">
+        <v>100000</v>
+      </c>
+      <c r="F22" s="20" t="n">
+        <v>120000</v>
+      </c>
+      <c r="G22" s="20" t="n">
+        <v>140000</v>
+      </c>
+      <c r="H22" s="15" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C23" s="21" t="n">
-        <v>0.015</v>
+        <v>62</v>
+      </c>
+      <c r="C23" s="20" t="n">
+        <v>4</v>
       </c>
       <c r="H23" s="15"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B24" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C24" s="19" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="H24" s="15" t="s">
-        <v>73</v>
-      </c>
+      <c r="C24" s="21" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="H24" s="15"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
@@ -2261,8 +2270,8 @@
       <c r="B25" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C25" s="21" t="n">
-        <v>0.005</v>
+      <c r="C25" s="19" t="n">
+        <v>0.4</v>
       </c>
       <c r="H25" s="15" t="s">
         <v>75</v>
@@ -2275,20 +2284,8 @@
       <c r="B26" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C26" s="19" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="D26" s="19" t="n">
-        <v>0.035</v>
-      </c>
-      <c r="E26" s="19" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="F26" s="19" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="G26" s="19" t="n">
-        <v>0.03</v>
+      <c r="C26" s="21" t="n">
+        <v>0.005</v>
       </c>
       <c r="H26" s="15" t="s">
         <v>77</v>
@@ -2302,7 +2299,19 @@
         <v>20</v>
       </c>
       <c r="C27" s="19" t="n">
-        <v>0.5</v>
+        <v>0.04</v>
+      </c>
+      <c r="D27" s="19" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="E27" s="19" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="F27" s="19" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="G27" s="19" t="n">
+        <v>0.03</v>
       </c>
       <c r="H27" s="15" t="s">
         <v>79</v>
@@ -2313,62 +2322,62 @@
         <v>80</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="C28" s="20" t="n">
-        <v>500</v>
+        <v>20</v>
+      </c>
+      <c r="C28" s="19" t="n">
+        <v>0.5</v>
       </c>
       <c r="H28" s="15" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="11" t="s">
+      <c r="A29" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="B29" s="12"/>
-      <c r="C29" s="12"/>
-      <c r="D29" s="12"/>
-      <c r="E29" s="12"/>
-      <c r="F29" s="12"/>
-      <c r="G29" s="12"/>
-      <c r="H29" s="12"/>
+      <c r="B29" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C29" s="20" t="n">
+        <v>500</v>
+      </c>
+      <c r="H29" s="15" t="s">
+        <v>83</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="B30" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="C30" s="18" t="n">
-        <v>20000</v>
-      </c>
-      <c r="D30" s="18" t="n">
-        <v>22000</v>
-      </c>
-      <c r="E30" s="18" t="n">
-        <v>25000</v>
-      </c>
-      <c r="F30" s="18" t="n">
-        <v>27000</v>
-      </c>
-      <c r="G30" s="18" t="n">
-        <v>30000</v>
-      </c>
-      <c r="H30" s="15" t="s">
+      <c r="A30" s="11" t="s">
         <v>84</v>
       </c>
+      <c r="B30" s="12"/>
+      <c r="C30" s="12"/>
+      <c r="D30" s="12"/>
+      <c r="E30" s="12"/>
+      <c r="F30" s="12"/>
+      <c r="G30" s="12"/>
+      <c r="H30" s="12"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="6" t="s">
         <v>85</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C31" s="21" t="n">
-        <v>0.45</v>
+        <v>25</v>
+      </c>
+      <c r="C31" s="18" t="n">
+        <v>20000</v>
+      </c>
+      <c r="D31" s="18" t="n">
+        <v>22000</v>
+      </c>
+      <c r="E31" s="18" t="n">
+        <v>25000</v>
+      </c>
+      <c r="F31" s="18" t="n">
+        <v>27000</v>
+      </c>
+      <c r="G31" s="18" t="n">
+        <v>30000</v>
       </c>
       <c r="H31" s="15" t="s">
         <v>86</v>
@@ -2382,7 +2391,7 @@
         <v>20</v>
       </c>
       <c r="C32" s="21" t="n">
-        <v>0.1</v>
+        <v>0.45</v>
       </c>
       <c r="H32" s="15" t="s">
         <v>88</v>
@@ -2393,22 +2402,10 @@
         <v>89</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="C33" s="18" t="n">
-        <v>25000</v>
-      </c>
-      <c r="D33" s="18" t="n">
-        <v>30000</v>
-      </c>
-      <c r="E33" s="18" t="n">
-        <v>35000</v>
-      </c>
-      <c r="F33" s="18" t="n">
-        <v>40000</v>
-      </c>
-      <c r="G33" s="18" t="n">
-        <v>45000</v>
+        <v>20</v>
+      </c>
+      <c r="C33" s="21" t="n">
+        <v>0.1</v>
       </c>
       <c r="H33" s="15" t="s">
         <v>90</v>
@@ -2419,22 +2416,22 @@
         <v>91</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C34" s="21" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="D34" s="21" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="E34" s="21" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="F34" s="21" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="G34" s="21" t="n">
-        <v>0.2</v>
+        <v>25</v>
+      </c>
+      <c r="C34" s="18" t="n">
+        <v>25000</v>
+      </c>
+      <c r="D34" s="18" t="n">
+        <v>30000</v>
+      </c>
+      <c r="E34" s="18" t="n">
+        <v>35000</v>
+      </c>
+      <c r="F34" s="18" t="n">
+        <v>40000</v>
+      </c>
+      <c r="G34" s="18" t="n">
+        <v>45000</v>
       </c>
       <c r="H34" s="15" t="s">
         <v>92</v>
@@ -2448,47 +2445,59 @@
         <v>20</v>
       </c>
       <c r="C35" s="21" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="H35" s="15"/>
+        <v>0.15</v>
+      </c>
+      <c r="D35" s="21" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="E35" s="21" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F35" s="21" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G35" s="21" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H35" s="15" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="6" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B36" s="6" t="s">
         <v>20</v>
       </c>
       <c r="C36" s="21" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="H36" s="15"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C37" s="21" t="n">
         <v>0.15</v>
       </c>
-      <c r="H36" s="15"/>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="11" t="s">
-        <v>95</v>
-      </c>
-      <c r="B37" s="12"/>
-      <c r="C37" s="12"/>
-      <c r="D37" s="12"/>
-      <c r="E37" s="12"/>
-      <c r="F37" s="12"/>
-      <c r="G37" s="12"/>
-      <c r="H37" s="12"/>
+      <c r="H37" s="15"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="B38" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C38" s="19" t="n">
-        <v>0.015</v>
-      </c>
-      <c r="H38" s="15" t="s">
+      <c r="A38" s="11" t="s">
         <v>97</v>
       </c>
+      <c r="B38" s="12"/>
+      <c r="C38" s="12"/>
+      <c r="D38" s="12"/>
+      <c r="E38" s="12"/>
+      <c r="F38" s="12"/>
+      <c r="G38" s="12"/>
+      <c r="H38" s="12"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="6" t="s">
@@ -2497,112 +2506,100 @@
       <c r="B39" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C39" s="21" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="H39" s="15"/>
+      <c r="C39" s="19" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="H39" s="15" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B40" s="6" t="s">
         <v>20</v>
       </c>
       <c r="C40" s="21" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="H40" s="15"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="C41" s="18" t="n">
-        <v>1000</v>
+        <v>20</v>
+      </c>
+      <c r="C41" s="21" t="n">
+        <v>0.02</v>
       </c>
       <c r="H41" s="15"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C42" s="19" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="H42" s="15" t="s">
-        <v>102</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="C42" s="18" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H42" s="15"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="6" t="s">
         <v>103</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="C43" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="D43" s="20" t="n">
-        <v>200</v>
-      </c>
-      <c r="E43" s="20" t="n">
-        <v>400</v>
-      </c>
-      <c r="F43" s="20" t="n">
-        <v>600</v>
-      </c>
-      <c r="G43" s="20" t="n">
-        <v>800</v>
+        <v>20</v>
+      </c>
+      <c r="C43" s="19" t="n">
+        <v>0.03</v>
       </c>
       <c r="H43" s="15" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="11" t="s">
+      <c r="A44" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="B44" s="12"/>
-      <c r="C44" s="12"/>
-      <c r="D44" s="12"/>
-      <c r="E44" s="12"/>
-      <c r="F44" s="12"/>
-      <c r="G44" s="12"/>
-      <c r="H44" s="12"/>
+      <c r="B44" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C44" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="D44" s="20" t="n">
+        <v>200</v>
+      </c>
+      <c r="E44" s="20" t="n">
+        <v>400</v>
+      </c>
+      <c r="F44" s="20" t="n">
+        <v>600</v>
+      </c>
+      <c r="G44" s="20" t="n">
+        <v>800</v>
+      </c>
+      <c r="H44" s="15" t="s">
+        <v>106</v>
+      </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="B45" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C45" s="19" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="D45" s="19" t="n">
-        <v>0.009</v>
-      </c>
-      <c r="E45" s="19" t="n">
-        <v>0.008</v>
-      </c>
-      <c r="F45" s="19" t="n">
-        <v>0.008</v>
-      </c>
-      <c r="G45" s="19" t="n">
-        <v>0.007</v>
-      </c>
-      <c r="H45" s="15" t="s">
+      <c r="A45" s="11" t="s">
         <v>107</v>
       </c>
+      <c r="B45" s="12"/>
+      <c r="C45" s="12"/>
+      <c r="D45" s="12"/>
+      <c r="E45" s="12"/>
+      <c r="F45" s="12"/>
+      <c r="G45" s="12"/>
+      <c r="H45" s="12"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="6" t="s">
@@ -2612,19 +2609,19 @@
         <v>20</v>
       </c>
       <c r="C46" s="19" t="n">
-        <v>0.006</v>
+        <v>0.01</v>
       </c>
       <c r="D46" s="19" t="n">
-        <v>0.005</v>
+        <v>0.009</v>
       </c>
       <c r="E46" s="19" t="n">
-        <v>0.005</v>
+        <v>0.008</v>
       </c>
       <c r="F46" s="19" t="n">
-        <v>0.004</v>
+        <v>0.008</v>
       </c>
       <c r="G46" s="19" t="n">
-        <v>0.004</v>
+        <v>0.007</v>
       </c>
       <c r="H46" s="15" t="s">
         <v>109</v>
@@ -2635,138 +2632,138 @@
         <v>110</v>
       </c>
       <c r="B47" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C47" s="19" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="D47" s="19" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="E47" s="19" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="F47" s="19" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="G47" s="19" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="H47" s="15" t="s">
         <v>111</v>
-      </c>
-      <c r="C47" s="20" t="n">
-        <v>2</v>
-      </c>
-      <c r="H47" s="15" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="B48" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="B48" s="6" t="s">
-        <v>25</v>
-      </c>
       <c r="C48" s="20" t="n">
-        <v>15</v>
-      </c>
-      <c r="H48" s="15"/>
+        <v>2</v>
+      </c>
+      <c r="H48" s="15" t="s">
+        <v>114</v>
+      </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="6" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C49" s="21" t="n">
-        <v>0.4</v>
+        <v>25</v>
+      </c>
+      <c r="C49" s="20" t="n">
+        <v>15</v>
       </c>
       <c r="H49" s="15"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="6" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B50" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="C50" s="20" t="n">
-        <v>300</v>
-      </c>
-      <c r="H50" s="15" t="s">
-        <v>116</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="C50" s="21" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H50" s="15"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="6" t="s">
         <v>117</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C51" s="21" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="H51" s="15"/>
+        <v>25</v>
+      </c>
+      <c r="C51" s="20" t="n">
+        <v>300</v>
+      </c>
+      <c r="H51" s="15" t="s">
+        <v>118</v>
+      </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B52" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C52" s="21" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="H52" s="15"/>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="B53" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C52" s="20" t="n">
+      <c r="C53" s="20" t="n">
         <v>500</v>
       </c>
-      <c r="H52" s="15" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="11" t="s">
-        <v>120</v>
-      </c>
-      <c r="B53" s="12"/>
-      <c r="C53" s="12"/>
-      <c r="D53" s="12"/>
-      <c r="E53" s="12"/>
-      <c r="F53" s="12"/>
-      <c r="G53" s="12"/>
-      <c r="H53" s="12"/>
+      <c r="H53" s="15" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="6" t="s">
-        <v>121</v>
-      </c>
-      <c r="B54" s="6" t="s">
+      <c r="A54" s="11" t="s">
         <v>122</v>
       </c>
-      <c r="C54" s="18" t="n">
-        <v>8</v>
-      </c>
-      <c r="D54" s="18" t="n">
-        <v>14</v>
-      </c>
-      <c r="E54" s="18" t="n">
-        <v>22</v>
-      </c>
-      <c r="F54" s="18" t="n">
-        <v>32</v>
-      </c>
-      <c r="G54" s="18" t="n">
-        <v>42</v>
-      </c>
-      <c r="H54" s="15" t="s">
-        <v>123</v>
-      </c>
+      <c r="B54" s="12"/>
+      <c r="C54" s="12"/>
+      <c r="D54" s="12"/>
+      <c r="E54" s="12"/>
+      <c r="F54" s="12"/>
+      <c r="G54" s="12"/>
+      <c r="H54" s="12"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="B55" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="B55" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="C55" s="20" t="n">
-        <v>7200000</v>
-      </c>
-      <c r="D55" s="20" t="n">
-        <v>7560000</v>
-      </c>
-      <c r="E55" s="20" t="n">
-        <v>7938000</v>
-      </c>
-      <c r="F55" s="20" t="n">
-        <v>8335000</v>
-      </c>
-      <c r="G55" s="20" t="n">
-        <v>8752000</v>
+      <c r="C55" s="18" t="n">
+        <v>8</v>
+      </c>
+      <c r="D55" s="18" t="n">
+        <v>14</v>
+      </c>
+      <c r="E55" s="18" t="n">
+        <v>22</v>
+      </c>
+      <c r="F55" s="18" t="n">
+        <v>32</v>
+      </c>
+      <c r="G55" s="18" t="n">
+        <v>42</v>
       </c>
       <c r="H55" s="15" t="s">
         <v>125</v>
@@ -2779,20 +2776,20 @@
       <c r="B56" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C56" s="18" t="n">
-        <v>1500</v>
-      </c>
-      <c r="D56" s="18" t="n">
-        <v>1300</v>
-      </c>
-      <c r="E56" s="18" t="n">
-        <v>1200</v>
-      </c>
-      <c r="F56" s="18" t="n">
-        <v>1100</v>
-      </c>
-      <c r="G56" s="18" t="n">
-        <v>1000</v>
+      <c r="C56" s="20" t="n">
+        <v>7200000</v>
+      </c>
+      <c r="D56" s="20" t="n">
+        <v>7560000</v>
+      </c>
+      <c r="E56" s="20" t="n">
+        <v>7938000</v>
+      </c>
+      <c r="F56" s="20" t="n">
+        <v>8335000</v>
+      </c>
+      <c r="G56" s="20" t="n">
+        <v>8752000</v>
       </c>
       <c r="H56" s="15" t="s">
         <v>127</v>
@@ -2805,84 +2802,84 @@
       <c r="B57" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C57" s="20" t="n">
-        <v>15000000</v>
-      </c>
-      <c r="D57" s="20" t="n">
-        <v>30000000</v>
-      </c>
-      <c r="E57" s="20" t="n">
-        <v>50000000</v>
-      </c>
-      <c r="F57" s="20" t="n">
-        <v>70000000</v>
-      </c>
-      <c r="G57" s="20" t="n">
-        <v>90000000</v>
-      </c>
-      <c r="H57" s="15"/>
+      <c r="C57" s="18" t="n">
+        <v>1500</v>
+      </c>
+      <c r="D57" s="18" t="n">
+        <v>1300</v>
+      </c>
+      <c r="E57" s="18" t="n">
+        <v>1200</v>
+      </c>
+      <c r="F57" s="18" t="n">
+        <v>1100</v>
+      </c>
+      <c r="G57" s="18" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H57" s="15" t="s">
+        <v>129</v>
+      </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B58" s="6" t="s">
         <v>25</v>
       </c>
       <c r="C58" s="20" t="n">
-        <v>6000000</v>
+        <v>15000000</v>
       </c>
       <c r="D58" s="20" t="n">
-        <v>9000000</v>
+        <v>30000000</v>
       </c>
       <c r="E58" s="20" t="n">
-        <v>15000000</v>
+        <v>50000000</v>
       </c>
       <c r="F58" s="20" t="n">
-        <v>22000000</v>
+        <v>70000000</v>
       </c>
       <c r="G58" s="20" t="n">
-        <v>30000000</v>
+        <v>90000000</v>
       </c>
       <c r="H58" s="15"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B59" s="6" t="s">
         <v>25</v>
       </c>
       <c r="C59" s="20" t="n">
-        <v>120</v>
+        <v>6000000</v>
+      </c>
+      <c r="D59" s="20" t="n">
+        <v>9000000</v>
+      </c>
+      <c r="E59" s="20" t="n">
+        <v>15000000</v>
+      </c>
+      <c r="F59" s="20" t="n">
+        <v>22000000</v>
+      </c>
+      <c r="G59" s="20" t="n">
+        <v>30000000</v>
       </c>
       <c r="H59" s="15"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B60" s="6" t="s">
         <v>25</v>
       </c>
       <c r="C60" s="20" t="n">
-        <v>12000000</v>
-      </c>
-      <c r="D60" s="20" t="n">
-        <v>15000000</v>
-      </c>
-      <c r="E60" s="20" t="n">
-        <v>20000000</v>
-      </c>
-      <c r="F60" s="20" t="n">
-        <v>25000000</v>
-      </c>
-      <c r="G60" s="20" t="n">
-        <v>30000000</v>
-      </c>
-      <c r="H60" s="15" t="s">
-        <v>132</v>
-      </c>
+        <v>120</v>
+      </c>
+      <c r="H60" s="15"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="6" t="s">
@@ -2892,19 +2889,19 @@
         <v>25</v>
       </c>
       <c r="C61" s="20" t="n">
-        <v>10000000</v>
+        <v>12000000</v>
       </c>
       <c r="D61" s="20" t="n">
         <v>15000000</v>
       </c>
       <c r="E61" s="20" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="F61" s="20" t="n">
         <v>25000000</v>
       </c>
-      <c r="F61" s="20" t="n">
+      <c r="G61" s="20" t="n">
         <v>30000000</v>
-      </c>
-      <c r="G61" s="20" t="n">
-        <v>35000000</v>
       </c>
       <c r="H61" s="15" t="s">
         <v>134</v>
@@ -2918,48 +2915,74 @@
         <v>25</v>
       </c>
       <c r="C62" s="20" t="n">
-        <v>9000000</v>
+        <v>10000000</v>
       </c>
       <c r="D62" s="20" t="n">
-        <v>12000000</v>
+        <v>15000000</v>
       </c>
       <c r="E62" s="20" t="n">
-        <v>18000000</v>
+        <v>25000000</v>
       </c>
       <c r="F62" s="20" t="n">
-        <v>24000000</v>
+        <v>30000000</v>
       </c>
       <c r="G62" s="20" t="n">
-        <v>30000000</v>
-      </c>
-      <c r="H62" s="15"/>
+        <v>35000000</v>
+      </c>
+      <c r="H62" s="15" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="6" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C63" s="21" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="H63" s="15" t="s">
-        <v>137</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="C63" s="20" t="n">
+        <v>9000000</v>
+      </c>
+      <c r="D63" s="20" t="n">
+        <v>12000000</v>
+      </c>
+      <c r="E63" s="20" t="n">
+        <v>18000000</v>
+      </c>
+      <c r="F63" s="20" t="n">
+        <v>24000000</v>
+      </c>
+      <c r="G63" s="20" t="n">
+        <v>30000000</v>
+      </c>
+      <c r="H63" s="15"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="6" t="s">
         <v>138</v>
       </c>
       <c r="B64" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C64" s="21" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="H64" s="15" t="s">
         <v>139</v>
       </c>
-      <c r="C64" s="20" t="n">
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="B65" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="C65" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="H64" s="15" t="s">
-        <v>140</v>
+      <c r="H65" s="15" t="s">
+        <v>142</v>
       </c>
     </row>
   </sheetData>
@@ -2989,7 +3012,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3001,34 +3024,34 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B5" s="20" t="n">
         <v>25000000</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B6" s="20" t="n">
         <v>6000000</v>
@@ -3037,40 +3060,40 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B7" s="20" t="n">
         <v>5000000</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B8" s="20" t="n">
         <v>8000000</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B9" s="20" t="n">
         <v>6000000</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B10" s="20" t="n">
         <v>12000000</v>
@@ -3079,7 +3102,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B11" s="22" t="n">
         <f aca="false">SUM(B5:B10)</f>
@@ -3088,7 +3111,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B12" s="23" t="n">
         <v>3</v>
@@ -3121,7 +3144,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3133,12 +3156,12 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>3</v>
@@ -3159,7 +3182,7 @@
         <v>8</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3205,7 +3228,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>10</v>
@@ -3231,12 +3254,12 @@
         <v>525000</v>
       </c>
       <c r="H7" s="15" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>10</v>
@@ -3265,7 +3288,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>10</v>
@@ -3294,7 +3317,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>10</v>
@@ -3323,7 +3346,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12"/>
@@ -3341,177 +3364,179 @@
         <v>13</v>
       </c>
       <c r="C12" s="25" t="n">
-        <f aca="false">C9*Hypothèses!C30*12</f>
+        <f aca="false">C9*Hypothèses!C31*12</f>
         <v>1050000000</v>
       </c>
       <c r="D12" s="25" t="n">
-        <f aca="false">D9*Hypothèses!D30*12</f>
+        <f aca="false">D9*Hypothèses!D31*12</f>
         <v>6072000000</v>
       </c>
       <c r="E12" s="25" t="n">
-        <f aca="false">E9*Hypothèses!E30*12</f>
+        <f aca="false">E9*Hypothèses!E31*12</f>
         <v>20925000000</v>
       </c>
       <c r="F12" s="25" t="n">
-        <f aca="false">F9*Hypothèses!F30*12</f>
+        <f aca="false">F9*Hypothèses!F31*12</f>
         <v>48211200000</v>
       </c>
       <c r="G12" s="25" t="n">
-        <f aca="false">G9*Hypothèses!G30*12</f>
+        <f aca="false">G9*Hypothèses!G31*12</f>
         <v>94500000000</v>
       </c>
       <c r="H12" s="15" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B13" s="6" t="s">
         <v>13</v>
       </c>
       <c r="C13" s="25" t="n">
-        <f aca="false">C12*Hypothèses!$C$31</f>
+        <f aca="false">C12*Hypothèses!$C$32</f>
         <v>472500000</v>
       </c>
       <c r="D13" s="25" t="n">
-        <f aca="false">D12*Hypothèses!$C$31</f>
+        <f aca="false">D12*Hypothèses!$C$32</f>
         <v>2732400000</v>
       </c>
       <c r="E13" s="25" t="n">
-        <f aca="false">E12*Hypothèses!$C$31</f>
+        <f aca="false">E12*Hypothèses!$C$32</f>
         <v>9416250000</v>
       </c>
       <c r="F13" s="25" t="n">
-        <f aca="false">F12*Hypothèses!$C$31</f>
+        <f aca="false">F12*Hypothèses!$C$32</f>
         <v>21695040000</v>
       </c>
       <c r="G13" s="25" t="n">
-        <f aca="false">G12*Hypothèses!$C$31</f>
+        <f aca="false">G12*Hypothèses!$C$32</f>
         <v>42525000000</v>
       </c>
       <c r="H13" s="15"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>13</v>
       </c>
       <c r="C14" s="25" t="n">
-        <f aca="false">C13*(1-Hypothèses!$C$32)</f>
+        <f aca="false">MAX(0,C13*(1-Hypothèses!$C$33)-Hypothèses!C12*C9*Hypothèses!C11*12*Hypothèses!$C$14)</f>
         <v>425250000</v>
       </c>
       <c r="D14" s="25" t="n">
-        <f aca="false">D13*(1-Hypothèses!$C$32)</f>
+        <f aca="false">MAX(0,D13*(1-Hypothèses!$C$33)-Hypothèses!D12*D9*Hypothèses!D11*12*Hypothèses!$C$14)</f>
         <v>2459160000</v>
       </c>
       <c r="E14" s="25" t="n">
-        <f aca="false">E13*(1-Hypothèses!$C$32)</f>
+        <f aca="false">MAX(0,E13*(1-Hypothèses!$C$33)-Hypothèses!E12*E9*Hypothèses!E11*12*Hypothèses!$C$14)</f>
         <v>8474625000</v>
       </c>
       <c r="F14" s="25" t="n">
-        <f aca="false">F13*(1-Hypothèses!$C$32)</f>
+        <f aca="false">MAX(0,F13*(1-Hypothèses!$C$33)-Hypothèses!F12*F9*Hypothèses!F11*12*Hypothèses!$C$14)</f>
         <v>19525536000</v>
       </c>
       <c r="G14" s="25" t="n">
-        <f aca="false">G13*(1-Hypothèses!$C$32)</f>
+        <f aca="false">MAX(0,G13*(1-Hypothèses!$C$33)-Hypothèses!G12*G9*Hypothèses!G11*12*Hypothèses!$C$14)</f>
         <v>38272500000</v>
       </c>
-      <c r="H14" s="15"/>
+      <c r="H14" s="15" t="s">
+        <v>173</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="B15" s="6" t="s">
         <v>13</v>
       </c>
       <c r="C15" s="25" t="n">
-        <f aca="false">C9*Hypothèses!C33</f>
+        <f aca="false">C9*Hypothèses!C34</f>
         <v>109375000</v>
       </c>
       <c r="D15" s="25" t="n">
-        <f aca="false">D9*Hypothèses!D33</f>
+        <f aca="false">D9*Hypothèses!D34</f>
         <v>690000000</v>
       </c>
       <c r="E15" s="25" t="n">
-        <f aca="false">E9*Hypothèses!E33</f>
+        <f aca="false">E9*Hypothèses!E34</f>
         <v>2441250000</v>
       </c>
       <c r="F15" s="25" t="n">
-        <f aca="false">F9*Hypothèses!F33</f>
+        <f aca="false">F9*Hypothèses!F34</f>
         <v>5952000000</v>
       </c>
       <c r="G15" s="25" t="n">
-        <f aca="false">G9*Hypothèses!G33</f>
+        <f aca="false">G9*Hypothèses!G34</f>
         <v>11812500000</v>
       </c>
       <c r="H15" s="15"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="B16" s="6" t="s">
         <v>13</v>
       </c>
       <c r="C16" s="25" t="n">
-        <f aca="false">C12*Hypothèses!C34</f>
+        <f aca="false">C12*Hypothèses!C35</f>
         <v>157500000</v>
       </c>
       <c r="D16" s="25" t="n">
-        <f aca="false">D12*Hypothèses!D34</f>
+        <f aca="false">D12*Hypothèses!D35</f>
         <v>1092960000</v>
       </c>
       <c r="E16" s="25" t="n">
-        <f aca="false">E12*Hypothèses!E34</f>
+        <f aca="false">E12*Hypothèses!E35</f>
         <v>4185000000</v>
       </c>
       <c r="F16" s="25" t="n">
-        <f aca="false">F12*Hypothèses!F34</f>
+        <f aca="false">F12*Hypothèses!F35</f>
         <v>9642240000</v>
       </c>
       <c r="G16" s="25" t="n">
-        <f aca="false">G12*Hypothèses!G34</f>
+        <f aca="false">G12*Hypothèses!G35</f>
         <v>18900000000</v>
       </c>
       <c r="H16" s="15"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="B17" s="6" t="s">
         <v>13</v>
       </c>
       <c r="C17" s="25" t="n">
-        <f aca="false">C15*Hypothèses!$C$35*Hypothèses!$C$36</f>
+        <f aca="false">C15*Hypothèses!$C$36*Hypothèses!$C$37</f>
         <v>4921875</v>
       </c>
       <c r="D17" s="25" t="n">
-        <f aca="false">D15*Hypothèses!$C$35*Hypothèses!$C$36</f>
+        <f aca="false">D15*Hypothèses!$C$36*Hypothèses!$C$37</f>
         <v>31050000</v>
       </c>
       <c r="E17" s="25" t="n">
-        <f aca="false">E15*Hypothèses!$C$35*Hypothèses!$C$36</f>
+        <f aca="false">E15*Hypothèses!$C$36*Hypothèses!$C$37</f>
         <v>109856250</v>
       </c>
       <c r="F17" s="25" t="n">
-        <f aca="false">F15*Hypothèses!$C$35*Hypothèses!$C$36</f>
+        <f aca="false">F15*Hypothèses!$C$36*Hypothèses!$C$37</f>
         <v>267840000</v>
       </c>
       <c r="G17" s="25" t="n">
-        <f aca="false">G15*Hypothèses!$C$35*Hypothèses!$C$36</f>
+        <f aca="false">G15*Hypothèses!$C$36*Hypothèses!$C$37</f>
         <v>531562500</v>
       </c>
       <c r="H17" s="15"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>10</v>
@@ -3566,99 +3591,99 @@
         <v>66150000000</v>
       </c>
       <c r="H19" s="15" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="B20" s="6" t="s">
         <v>13</v>
       </c>
       <c r="C20" s="25" t="n">
-        <f aca="false">C18*Hypothèses!C15*Hypothèses!C16</f>
+        <f aca="false">C18*Hypothèses!C16*Hypothèses!C17</f>
         <v>7000000</v>
       </c>
       <c r="D20" s="25" t="n">
-        <f aca="false">D18*Hypothèses!D15*Hypothèses!D16</f>
+        <f aca="false">D18*Hypothèses!D16*Hypothèses!D17</f>
         <v>77625000</v>
       </c>
       <c r="E20" s="25" t="n">
-        <f aca="false">E18*Hypothèses!E15*Hypothèses!E16</f>
+        <f aca="false">E18*Hypothèses!E16*Hypothèses!E17</f>
         <v>383625000</v>
       </c>
       <c r="F20" s="25" t="n">
-        <f aca="false">F18*Hypothèses!F15*Hypothèses!F16</f>
+        <f aca="false">F18*Hypothèses!F16*Hypothèses!F17</f>
         <v>982080000</v>
       </c>
       <c r="G20" s="25" t="n">
-        <f aca="false">G18*Hypothèses!G15*Hypothèses!G16</f>
+        <f aca="false">G18*Hypothèses!G16*Hypothèses!G17</f>
         <v>1890000000</v>
       </c>
       <c r="H20" s="15"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C21" s="24" t="n">
-        <f aca="false">C9*Hypothèses!C19*Hypothèses!$C$20</f>
+        <f aca="false">C9*Hypothèses!C20*Hypothèses!$C$21</f>
         <v>87.5</v>
       </c>
       <c r="D21" s="24" t="n">
-        <f aca="false">D9*Hypothèses!D19*Hypothèses!$C$20</f>
+        <f aca="false">D9*Hypothèses!D20*Hypothèses!$C$21</f>
         <v>1380</v>
       </c>
       <c r="E21" s="24" t="n">
-        <f aca="false">E9*Hypothèses!E19*Hypothèses!$C$20</f>
+        <f aca="false">E9*Hypothèses!E20*Hypothèses!$C$21</f>
         <v>6975</v>
       </c>
       <c r="F21" s="24" t="n">
-        <f aca="false">F9*Hypothèses!F19*Hypothèses!$C$20</f>
+        <f aca="false">F9*Hypothèses!F20*Hypothèses!$C$21</f>
         <v>20832</v>
       </c>
       <c r="G21" s="24" t="n">
-        <f aca="false">G9*Hypothèses!G19*Hypothèses!$C$20</f>
+        <f aca="false">G9*Hypothèses!G20*Hypothèses!$C$21</f>
         <v>42000</v>
       </c>
       <c r="H21" s="15"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="B22" s="6" t="s">
         <v>13</v>
       </c>
       <c r="C22" s="25" t="n">
-        <f aca="false">C21*Hypothèses!C21</f>
+        <f aca="false">C21*Hypothèses!C22</f>
         <v>6562500</v>
       </c>
       <c r="D22" s="25" t="n">
-        <f aca="false">D21*Hypothèses!D21</f>
+        <f aca="false">D21*Hypothèses!D22</f>
         <v>124200000</v>
       </c>
       <c r="E22" s="25" t="n">
-        <f aca="false">E21*Hypothèses!E21</f>
+        <f aca="false">E21*Hypothèses!E22</f>
         <v>697500000</v>
       </c>
       <c r="F22" s="25" t="n">
-        <f aca="false">F21*Hypothèses!F21</f>
+        <f aca="false">F21*Hypothèses!F22</f>
         <v>2499840000</v>
       </c>
       <c r="G22" s="25" t="n">
-        <f aca="false">G21*Hypothèses!G21</f>
+        <f aca="false">G21*Hypothèses!G22</f>
         <v>5880000000</v>
       </c>
       <c r="H22" s="15"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="B23" s="6" t="s">
         <v>13</v>
@@ -3687,38 +3712,38 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="B24" s="6" t="s">
         <v>13</v>
       </c>
       <c r="C24" s="25" t="n">
-        <f aca="false">C20*Hypothèses!$C$18*Hypothèses!$C$17+C22*Hypothèses!$C$23*(Hypothèses!$C$22+1)/2</f>
+        <f aca="false">C20*Hypothèses!$C$19*Hypothèses!$C$18+C22*Hypothèses!$C$24*(Hypothèses!$C$23+1)/2</f>
         <v>456093.75</v>
       </c>
       <c r="D24" s="25" t="n">
-        <f aca="false">D20*Hypothèses!$C$18*Hypothèses!$C$17+D22*Hypothèses!$C$23*(Hypothèses!$C$22+1)/2</f>
+        <f aca="false">D20*Hypothèses!$C$19*Hypothèses!$C$18+D22*Hypothèses!$C$24*(Hypothèses!$C$23+1)/2</f>
         <v>6986250</v>
       </c>
       <c r="E24" s="25" t="n">
-        <f aca="false">E20*Hypothèses!$C$18*Hypothèses!$C$17+E22*Hypothèses!$C$23*(Hypothèses!$C$22+1)/2</f>
+        <f aca="false">E20*Hypothèses!$C$19*Hypothèses!$C$18+E22*Hypothèses!$C$24*(Hypothèses!$C$23+1)/2</f>
         <v>37665000</v>
       </c>
       <c r="F24" s="25" t="n">
-        <f aca="false">F20*Hypothèses!$C$18*Hypothèses!$C$17+F22*Hypothèses!$C$23*(Hypothèses!$C$22+1)/2</f>
+        <f aca="false">F20*Hypothèses!$C$19*Hypothèses!$C$18+F22*Hypothèses!$C$24*(Hypothèses!$C$23+1)/2</f>
         <v>123206400</v>
       </c>
       <c r="G24" s="25" t="n">
-        <f aca="false">G20*Hypothèses!$C$18*Hypothèses!$C$17+G22*Hypothèses!$C$23*(Hypothèses!$C$22+1)/2</f>
+        <f aca="false">G20*Hypothèses!$C$19*Hypothèses!$C$18+G22*Hypothèses!$C$24*(Hypothèses!$C$23+1)/2</f>
         <v>277200000</v>
       </c>
       <c r="H24" s="15" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="11" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="12"/>
@@ -3730,7 +3755,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="B26" s="6" t="s">
         <v>13</v>
@@ -3759,203 +3784,203 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="B27" s="6" t="s">
         <v>13</v>
       </c>
       <c r="C27" s="25" t="n">
-        <f aca="false">C24*Hypothèses!$C$24</f>
+        <f aca="false">C24*Hypothèses!$C$25</f>
         <v>182437.5</v>
       </c>
       <c r="D27" s="25" t="n">
-        <f aca="false">D24*Hypothèses!$C$24</f>
+        <f aca="false">D24*Hypothèses!$C$25</f>
         <v>2794500</v>
       </c>
       <c r="E27" s="25" t="n">
-        <f aca="false">E24*Hypothèses!$C$24</f>
+        <f aca="false">E24*Hypothèses!$C$25</f>
         <v>15066000</v>
       </c>
       <c r="F27" s="25" t="n">
-        <f aca="false">F24*Hypothèses!$C$24</f>
+        <f aca="false">F24*Hypothèses!$C$25</f>
         <v>49282560</v>
       </c>
       <c r="G27" s="25" t="n">
-        <f aca="false">G24*Hypothèses!$C$24</f>
+        <f aca="false">G24*Hypothèses!$C$25</f>
         <v>110880000</v>
       </c>
       <c r="H27" s="15"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B28" s="6" t="s">
         <v>13</v>
       </c>
       <c r="C28" s="25" t="n">
-        <f aca="false">C14*Hypothèses!$C$38</f>
+        <f aca="false">C14*Hypothèses!$C$39</f>
         <v>6378750</v>
       </c>
       <c r="D28" s="25" t="n">
-        <f aca="false">D14*Hypothèses!$C$38</f>
+        <f aca="false">D14*Hypothèses!$C$39</f>
         <v>36887400</v>
       </c>
       <c r="E28" s="25" t="n">
-        <f aca="false">E14*Hypothèses!$C$38</f>
+        <f aca="false">E14*Hypothèses!$C$39</f>
         <v>127119375</v>
       </c>
       <c r="F28" s="25" t="n">
-        <f aca="false">F14*Hypothèses!$C$38</f>
+        <f aca="false">F14*Hypothèses!$C$39</f>
         <v>292883040</v>
       </c>
       <c r="G28" s="25" t="n">
-        <f aca="false">G14*Hypothèses!$C$38</f>
+        <f aca="false">G14*Hypothèses!$C$39</f>
         <v>574087500</v>
       </c>
       <c r="H28" s="15"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="B29" s="6" t="s">
         <v>13</v>
       </c>
       <c r="C29" s="25" t="n">
-        <f aca="false">C16*Hypothèses!$C$39</f>
+        <f aca="false">C16*Hypothèses!$C$40</f>
         <v>1575000</v>
       </c>
       <c r="D29" s="25" t="n">
-        <f aca="false">D16*Hypothèses!$C$39</f>
+        <f aca="false">D16*Hypothèses!$C$40</f>
         <v>10929600</v>
       </c>
       <c r="E29" s="25" t="n">
-        <f aca="false">E16*Hypothèses!$C$39</f>
+        <f aca="false">E16*Hypothèses!$C$40</f>
         <v>41850000</v>
       </c>
       <c r="F29" s="25" t="n">
-        <f aca="false">F16*Hypothèses!$C$39</f>
+        <f aca="false">F16*Hypothèses!$C$40</f>
         <v>96422400</v>
       </c>
       <c r="G29" s="25" t="n">
-        <f aca="false">G16*Hypothèses!$C$39</f>
+        <f aca="false">G16*Hypothèses!$C$40</f>
         <v>189000000</v>
       </c>
       <c r="H29" s="15"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="B30" s="6" t="s">
         <v>13</v>
       </c>
       <c r="C30" s="25" t="n">
-        <f aca="false">C17*Hypothèses!$C$40</f>
+        <f aca="false">C17*Hypothèses!$C$41</f>
         <v>98437.5</v>
       </c>
       <c r="D30" s="25" t="n">
-        <f aca="false">D17*Hypothèses!$C$40</f>
+        <f aca="false">D17*Hypothèses!$C$41</f>
         <v>621000</v>
       </c>
       <c r="E30" s="25" t="n">
-        <f aca="false">E17*Hypothèses!$C$40</f>
+        <f aca="false">E17*Hypothèses!$C$41</f>
         <v>2197125</v>
       </c>
       <c r="F30" s="25" t="n">
-        <f aca="false">F17*Hypothèses!$C$40</f>
+        <f aca="false">F17*Hypothèses!$C$41</f>
         <v>5356800</v>
       </c>
       <c r="G30" s="25" t="n">
-        <f aca="false">G17*Hypothèses!$C$40</f>
+        <f aca="false">G17*Hypothèses!$C$41</f>
         <v>10631250</v>
       </c>
       <c r="H30" s="15"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="6" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="B31" s="6" t="s">
         <v>13</v>
       </c>
       <c r="C31" s="25" t="n">
-        <f aca="false">C10*Hypothèses!$C$41*12</f>
+        <f aca="false">C10*Hypothèses!$C$42*12</f>
         <v>1575000</v>
       </c>
       <c r="D31" s="25" t="n">
-        <f aca="false">D10*Hypothèses!$C$41*12</f>
+        <f aca="false">D10*Hypothèses!$C$42*12</f>
         <v>13800000</v>
       </c>
       <c r="E31" s="25" t="n">
-        <f aca="false">E10*Hypothèses!$C$41*12</f>
+        <f aca="false">E10*Hypothèses!$C$42*12</f>
         <v>58590000</v>
       </c>
       <c r="F31" s="25" t="n">
-        <f aca="false">F10*Hypothèses!$C$41*12</f>
+        <f aca="false">F10*Hypothèses!$C$42*12</f>
         <v>142848000</v>
       </c>
       <c r="G31" s="25" t="n">
-        <f aca="false">G10*Hypothèses!$C$41*12</f>
+        <f aca="false">G10*Hypothèses!$C$42*12</f>
         <v>283500000</v>
       </c>
       <c r="H31" s="15"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="B32" s="6" t="s">
         <v>13</v>
       </c>
       <c r="C32" s="25" t="n">
-        <f aca="false">C15*Hypothèses!$C$42</f>
+        <f aca="false">C15*Hypothèses!$C$43</f>
         <v>3281250</v>
       </c>
       <c r="D32" s="25" t="n">
-        <f aca="false">D15*Hypothèses!$C$42</f>
+        <f aca="false">D15*Hypothèses!$C$43</f>
         <v>20700000</v>
       </c>
       <c r="E32" s="25" t="n">
-        <f aca="false">E15*Hypothèses!$C$42</f>
+        <f aca="false">E15*Hypothèses!$C$43</f>
         <v>73237500</v>
       </c>
       <c r="F32" s="25" t="n">
-        <f aca="false">F15*Hypothèses!$C$42</f>
+        <f aca="false">F15*Hypothèses!$C$43</f>
         <v>178560000</v>
       </c>
       <c r="G32" s="25" t="n">
-        <f aca="false">G15*Hypothèses!$C$42</f>
+        <f aca="false">G15*Hypothèses!$C$43</f>
         <v>354375000</v>
       </c>
       <c r="H32" s="15"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="6" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="B33" s="6" t="s">
         <v>13</v>
       </c>
       <c r="C33" s="25" t="n">
-        <f aca="false">C9*Hypothèses!C43</f>
+        <f aca="false">C9*Hypothèses!C44</f>
         <v>0</v>
       </c>
       <c r="D33" s="25" t="n">
-        <f aca="false">D9*Hypothèses!D43</f>
+        <f aca="false">D9*Hypothèses!D44</f>
         <v>4600000</v>
       </c>
       <c r="E33" s="25" t="n">
-        <f aca="false">E9*Hypothèses!E43</f>
+        <f aca="false">E9*Hypothèses!E44</f>
         <v>27900000</v>
       </c>
       <c r="F33" s="25" t="n">
-        <f aca="false">F9*Hypothèses!F43</f>
+        <f aca="false">F9*Hypothèses!F44</f>
         <v>89280000</v>
       </c>
       <c r="G33" s="25" t="n">
-        <f aca="false">G9*Hypothèses!G43</f>
+        <f aca="false">G9*Hypothèses!G44</f>
         <v>210000000</v>
       </c>
       <c r="H33" s="15"/>
@@ -3991,7 +4016,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="11" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B35" s="12"/>
       <c r="C35" s="12"/>
@@ -4003,210 +4028,210 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="6" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="B36" s="6" t="s">
         <v>13</v>
       </c>
       <c r="C36" s="25" t="n">
-        <f aca="false">C12*Hypothèses!C45</f>
+        <f aca="false">C12*Hypothèses!C46</f>
         <v>10500000</v>
       </c>
       <c r="D36" s="25" t="n">
-        <f aca="false">D12*Hypothèses!D45</f>
+        <f aca="false">D12*Hypothèses!D46</f>
         <v>54648000</v>
       </c>
       <c r="E36" s="25" t="n">
-        <f aca="false">E12*Hypothèses!E45</f>
+        <f aca="false">E12*Hypothèses!E46</f>
         <v>167400000</v>
       </c>
       <c r="F36" s="25" t="n">
-        <f aca="false">F12*Hypothèses!F45</f>
+        <f aca="false">F12*Hypothèses!F46</f>
         <v>385689600</v>
       </c>
       <c r="G36" s="25" t="n">
-        <f aca="false">G12*Hypothèses!G45</f>
+        <f aca="false">G12*Hypothèses!G46</f>
         <v>661500000</v>
       </c>
       <c r="H36" s="15"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="6" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="B37" s="6" t="s">
         <v>13</v>
       </c>
       <c r="C37" s="25" t="n">
-        <f aca="false">C13*Hypothèses!C46</f>
+        <f aca="false">C13*Hypothèses!C47</f>
         <v>2835000</v>
       </c>
       <c r="D37" s="25" t="n">
-        <f aca="false">D13*Hypothèses!D46</f>
+        <f aca="false">D13*Hypothèses!D47</f>
         <v>13662000</v>
       </c>
       <c r="E37" s="25" t="n">
-        <f aca="false">E13*Hypothèses!E46</f>
+        <f aca="false">E13*Hypothèses!E47</f>
         <v>47081250</v>
       </c>
       <c r="F37" s="25" t="n">
-        <f aca="false">F13*Hypothèses!F46</f>
+        <f aca="false">F13*Hypothèses!F47</f>
         <v>86780160</v>
       </c>
       <c r="G37" s="25" t="n">
-        <f aca="false">G13*Hypothèses!G46</f>
+        <f aca="false">G13*Hypothèses!G47</f>
         <v>170100000</v>
       </c>
       <c r="H37" s="15"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="6" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="B38" s="6" t="s">
         <v>13</v>
       </c>
       <c r="C38" s="25" t="n">
-        <f aca="false">C9*Hypothèses!$C$47*12*Hypothèses!$C$48</f>
+        <f aca="false">C9*Hypothèses!$C$48*12*Hypothèses!$C$49</f>
         <v>1575000</v>
       </c>
       <c r="D38" s="25" t="n">
-        <f aca="false">D9*Hypothèses!$C$47*12*Hypothèses!$C$48</f>
+        <f aca="false">D9*Hypothèses!$C$48*12*Hypothèses!$C$49</f>
         <v>8280000</v>
       </c>
       <c r="E38" s="25" t="n">
-        <f aca="false">E9*Hypothèses!$C$47*12*Hypothèses!$C$48</f>
+        <f aca="false">E9*Hypothèses!$C$48*12*Hypothèses!$C$49</f>
         <v>25110000</v>
       </c>
       <c r="F38" s="25" t="n">
-        <f aca="false">F9*Hypothèses!$C$47*12*Hypothèses!$C$48</f>
+        <f aca="false">F9*Hypothèses!$C$48*12*Hypothèses!$C$49</f>
         <v>53568000</v>
       </c>
       <c r="G38" s="25" t="n">
-        <f aca="false">G9*Hypothèses!$C$47*12*Hypothèses!$C$48</f>
+        <f aca="false">G9*Hypothèses!$C$48*12*Hypothèses!$C$49</f>
         <v>94500000</v>
       </c>
       <c r="H38" s="15"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="6" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="B39" s="6" t="s">
         <v>13</v>
       </c>
       <c r="C39" s="25" t="n">
-        <f aca="false">C8*Hypothèses!$C$49*Hypothèses!$C$50</f>
+        <f aca="false">C8*Hypothèses!$C$50*Hypothèses!$C$51</f>
         <v>3000000</v>
       </c>
       <c r="D39" s="25" t="n">
-        <f aca="false">D8*Hypothèses!$C$49*Hypothèses!$C$50</f>
+        <f aca="false">D8*Hypothèses!$C$50*Hypothèses!$C$51</f>
         <v>7800000</v>
       </c>
       <c r="E39" s="25" t="n">
-        <f aca="false">E8*Hypothèses!$C$49*Hypothèses!$C$50</f>
+        <f aca="false">E8*Hypothèses!$C$50*Hypothèses!$C$51</f>
         <v>15600000</v>
       </c>
       <c r="F39" s="25" t="n">
-        <f aca="false">F8*Hypothèses!$C$49*Hypothèses!$C$50</f>
+        <f aca="false">F8*Hypothèses!$C$50*Hypothèses!$C$51</f>
         <v>21600000</v>
       </c>
       <c r="G39" s="25" t="n">
-        <f aca="false">G8*Hypothèses!$C$49*Hypothèses!$C$50</f>
+        <f aca="false">G8*Hypothèses!$C$50*Hypothèses!$C$51</f>
         <v>30000000</v>
       </c>
       <c r="H39" s="15"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="6" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="B40" s="6" t="s">
         <v>13</v>
       </c>
       <c r="C40" s="25" t="n">
-        <f aca="false">C8*Hypothèses!$C$51*Hypothèses!$C$52</f>
+        <f aca="false">C8*Hypothèses!$C$52*Hypothèses!$C$53</f>
         <v>3750000</v>
       </c>
       <c r="D40" s="25" t="n">
-        <f aca="false">D8*Hypothèses!$C$51*Hypothèses!$C$52</f>
+        <f aca="false">D8*Hypothèses!$C$52*Hypothèses!$C$53</f>
         <v>9750000</v>
       </c>
       <c r="E40" s="25" t="n">
-        <f aca="false">E8*Hypothèses!$C$51*Hypothèses!$C$52</f>
+        <f aca="false">E8*Hypothèses!$C$52*Hypothèses!$C$53</f>
         <v>19500000</v>
       </c>
       <c r="F40" s="25" t="n">
-        <f aca="false">F8*Hypothèses!$C$51*Hypothèses!$C$52</f>
+        <f aca="false">F8*Hypothèses!$C$52*Hypothèses!$C$53</f>
         <v>27000000</v>
       </c>
       <c r="G40" s="25" t="n">
-        <f aca="false">G8*Hypothèses!$C$51*Hypothèses!$C$52</f>
+        <f aca="false">G8*Hypothèses!$C$52*Hypothèses!$C$53</f>
         <v>37500000</v>
       </c>
       <c r="H40" s="15"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="6" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B41" s="6" t="s">
         <v>13</v>
       </c>
       <c r="C41" s="25" t="n">
-        <f aca="false">(C20*Hypothèses!$C$25+C22*Hypothèses!C26)*Hypothèses!$C$27</f>
+        <f aca="false">(C20*Hypothèses!$C$26+C22*Hypothèses!C27)*Hypothèses!$C$28</f>
         <v>148750</v>
       </c>
       <c r="D41" s="25" t="n">
-        <f aca="false">(D20*Hypothèses!$C$25+D22*Hypothèses!D26)*Hypothèses!$C$27</f>
+        <f aca="false">(D20*Hypothèses!$C$26+D22*Hypothèses!D27)*Hypothèses!$C$28</f>
         <v>2367562.5</v>
       </c>
       <c r="E41" s="25" t="n">
-        <f aca="false">(E20*Hypothèses!$C$25+E22*Hypothèses!E26)*Hypothèses!$C$27</f>
+        <f aca="false">(E20*Hypothèses!$C$26+E22*Hypothèses!E27)*Hypothèses!$C$28</f>
         <v>11421562.5</v>
       </c>
       <c r="F41" s="25" t="n">
-        <f aca="false">(F20*Hypothèses!$C$25+F22*Hypothèses!F26)*Hypothèses!$C$27</f>
+        <f aca="false">(F20*Hypothèses!$C$26+F22*Hypothèses!F27)*Hypothèses!$C$28</f>
         <v>39952800</v>
       </c>
       <c r="G41" s="25" t="n">
-        <f aca="false">(G20*Hypothèses!$C$25+G22*Hypothèses!G26)*Hypothèses!$C$27</f>
+        <f aca="false">(G20*Hypothèses!$C$26+G22*Hypothèses!G27)*Hypothèses!$C$28</f>
         <v>92925000</v>
       </c>
       <c r="H41" s="15"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="6" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="B42" s="6" t="s">
         <v>13</v>
       </c>
       <c r="C42" s="25" t="n">
-        <f aca="false">(C21+C18*Hypothèses!C15)*Hypothèses!$C$28</f>
+        <f aca="false">(C21+C18*Hypothèses!C16)*Hypothèses!$C$29</f>
         <v>131250</v>
       </c>
       <c r="D42" s="25" t="n">
-        <f aca="false">(D21+D18*Hypothèses!D15)*Hypothèses!$C$28</f>
+        <f aca="false">(D21+D18*Hypothèses!D16)*Hypothèses!$C$29</f>
         <v>1552500</v>
       </c>
       <c r="E42" s="25" t="n">
-        <f aca="false">(E21+E18*Hypothèses!E15)*Hypothèses!$C$28</f>
+        <f aca="false">(E21+E18*Hypothèses!E16)*Hypothèses!$C$29</f>
         <v>7323750</v>
       </c>
       <c r="F42" s="25" t="n">
-        <f aca="false">(F21+F18*Hypothèses!F15)*Hypothèses!$C$28</f>
+        <f aca="false">(F21+F18*Hypothèses!F16)*Hypothèses!$C$29</f>
         <v>19344000</v>
       </c>
       <c r="G42" s="25" t="n">
-        <f aca="false">(G21+G18*Hypothèses!G15)*Hypothèses!$C$28</f>
+        <f aca="false">(G21+G18*Hypothèses!G16)*Hypothèses!$C$29</f>
         <v>36750000</v>
       </c>
       <c r="H42" s="15"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="13" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="B43" s="6" t="s">
         <v>13</v>
@@ -4293,7 +4318,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="11" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B46" s="12"/>
       <c r="C46" s="12"/>
@@ -4305,212 +4330,212 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="6" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B47" s="6" t="s">
         <v>13</v>
       </c>
       <c r="C47" s="8" t="n">
-        <f aca="false">Hypothèses!C54*Hypothèses!C55</f>
+        <f aca="false">Hypothèses!C55*Hypothèses!C56</f>
         <v>57600000</v>
       </c>
       <c r="D47" s="8" t="n">
-        <f aca="false">Hypothèses!D54*Hypothèses!D55</f>
+        <f aca="false">Hypothèses!D55*Hypothèses!D56</f>
         <v>105840000</v>
       </c>
       <c r="E47" s="8" t="n">
-        <f aca="false">Hypothèses!E54*Hypothèses!E55</f>
+        <f aca="false">Hypothèses!E55*Hypothèses!E56</f>
         <v>174636000</v>
       </c>
       <c r="F47" s="8" t="n">
-        <f aca="false">Hypothèses!F54*Hypothèses!F55</f>
+        <f aca="false">Hypothèses!F55*Hypothèses!F56</f>
         <v>266720000</v>
       </c>
       <c r="G47" s="8" t="n">
-        <f aca="false">Hypothèses!G54*Hypothèses!G55</f>
+        <f aca="false">Hypothèses!G55*Hypothèses!G56</f>
         <v>367584000</v>
       </c>
       <c r="H47" s="15"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="6" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="B48" s="6" t="s">
         <v>13</v>
       </c>
       <c r="C48" s="25" t="n">
-        <f aca="false">C8*Hypothèses!C56</f>
+        <f aca="false">C8*Hypothèses!C57</f>
         <v>37500000</v>
       </c>
       <c r="D48" s="25" t="n">
-        <f aca="false">D8*Hypothèses!D56</f>
+        <f aca="false">D8*Hypothèses!D57</f>
         <v>84500000</v>
       </c>
       <c r="E48" s="25" t="n">
-        <f aca="false">E8*Hypothèses!E56</f>
+        <f aca="false">E8*Hypothèses!E57</f>
         <v>156000000</v>
       </c>
       <c r="F48" s="25" t="n">
-        <f aca="false">F8*Hypothèses!F56</f>
+        <f aca="false">F8*Hypothèses!F57</f>
         <v>198000000</v>
       </c>
       <c r="G48" s="25" t="n">
-        <f aca="false">G8*Hypothèses!G56</f>
+        <f aca="false">G8*Hypothèses!G57</f>
         <v>250000000</v>
       </c>
       <c r="H48" s="15" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="6" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="B49" s="6" t="s">
         <v>13</v>
       </c>
       <c r="C49" s="8" t="n">
-        <f aca="false">Hypothèses!C57</f>
+        <f aca="false">Hypothèses!C58</f>
         <v>15000000</v>
       </c>
       <c r="D49" s="8" t="n">
-        <f aca="false">Hypothèses!D57</f>
+        <f aca="false">Hypothèses!D58</f>
         <v>30000000</v>
       </c>
       <c r="E49" s="8" t="n">
-        <f aca="false">Hypothèses!E57</f>
+        <f aca="false">Hypothèses!E58</f>
         <v>50000000</v>
       </c>
       <c r="F49" s="8" t="n">
-        <f aca="false">Hypothèses!F57</f>
+        <f aca="false">Hypothèses!F58</f>
         <v>70000000</v>
       </c>
       <c r="G49" s="8" t="n">
-        <f aca="false">Hypothèses!G57</f>
+        <f aca="false">Hypothèses!G58</f>
         <v>90000000</v>
       </c>
       <c r="H49" s="15"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="6" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="B50" s="6" t="s">
         <v>13</v>
       </c>
       <c r="C50" s="8" t="n">
-        <f aca="false">Hypothèses!C58+C9*Hypothèses!$C$59</f>
+        <f aca="false">Hypothèses!C59+C9*Hypothèses!$C$60</f>
         <v>6525000</v>
       </c>
       <c r="D50" s="8" t="n">
-        <f aca="false">Hypothèses!D58+D9*Hypothèses!$C$59</f>
+        <f aca="false">Hypothèses!D59+D9*Hypothèses!$C$60</f>
         <v>11760000</v>
       </c>
       <c r="E50" s="8" t="n">
-        <f aca="false">Hypothèses!E58+E9*Hypothèses!$C$59</f>
+        <f aca="false">Hypothèses!E59+E9*Hypothèses!$C$60</f>
         <v>23370000</v>
       </c>
       <c r="F50" s="8" t="n">
-        <f aca="false">Hypothèses!F58+F9*Hypothèses!$C$59</f>
+        <f aca="false">Hypothèses!F59+F9*Hypothèses!$C$60</f>
         <v>39856000</v>
       </c>
       <c r="G50" s="8" t="n">
-        <f aca="false">Hypothèses!G58+G9*Hypothèses!$C$59</f>
+        <f aca="false">Hypothèses!G59+G9*Hypothèses!$C$60</f>
         <v>61500000</v>
       </c>
       <c r="H50" s="15"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="6" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="B51" s="6" t="s">
         <v>13</v>
       </c>
       <c r="C51" s="8" t="n">
-        <f aca="false">Hypothèses!C60</f>
+        <f aca="false">Hypothèses!C61</f>
         <v>12000000</v>
       </c>
       <c r="D51" s="8" t="n">
-        <f aca="false">Hypothèses!D60</f>
+        <f aca="false">Hypothèses!D61</f>
         <v>15000000</v>
       </c>
       <c r="E51" s="8" t="n">
-        <f aca="false">Hypothèses!E60</f>
+        <f aca="false">Hypothèses!E61</f>
         <v>20000000</v>
       </c>
       <c r="F51" s="8" t="n">
-        <f aca="false">Hypothèses!F60</f>
+        <f aca="false">Hypothèses!F61</f>
         <v>25000000</v>
       </c>
       <c r="G51" s="8" t="n">
-        <f aca="false">Hypothèses!G60</f>
+        <f aca="false">Hypothèses!G61</f>
         <v>30000000</v>
       </c>
       <c r="H51" s="15"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="6" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="B52" s="6" t="s">
         <v>13</v>
       </c>
       <c r="C52" s="8" t="n">
-        <f aca="false">Hypothèses!C61</f>
+        <f aca="false">Hypothèses!C62</f>
         <v>10000000</v>
       </c>
       <c r="D52" s="8" t="n">
-        <f aca="false">Hypothèses!D61</f>
+        <f aca="false">Hypothèses!D62</f>
         <v>15000000</v>
       </c>
       <c r="E52" s="8" t="n">
-        <f aca="false">Hypothèses!E61</f>
+        <f aca="false">Hypothèses!E62</f>
         <v>25000000</v>
       </c>
       <c r="F52" s="8" t="n">
-        <f aca="false">Hypothèses!F61</f>
+        <f aca="false">Hypothèses!F62</f>
         <v>30000000</v>
       </c>
       <c r="G52" s="8" t="n">
-        <f aca="false">Hypothèses!G61</f>
+        <f aca="false">Hypothèses!G62</f>
         <v>35000000</v>
       </c>
       <c r="H52" s="15"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B53" s="6" t="s">
         <v>13</v>
       </c>
       <c r="C53" s="8" t="n">
-        <f aca="false">Hypothèses!C62</f>
+        <f aca="false">Hypothèses!C63</f>
         <v>9000000</v>
       </c>
       <c r="D53" s="8" t="n">
-        <f aca="false">Hypothèses!D62</f>
+        <f aca="false">Hypothèses!D63</f>
         <v>12000000</v>
       </c>
       <c r="E53" s="8" t="n">
-        <f aca="false">Hypothèses!E62</f>
+        <f aca="false">Hypothèses!E63</f>
         <v>18000000</v>
       </c>
       <c r="F53" s="8" t="n">
-        <f aca="false">Hypothèses!F62</f>
+        <f aca="false">Hypothèses!F63</f>
         <v>24000000</v>
       </c>
       <c r="G53" s="8" t="n">
-        <f aca="false">Hypothèses!G62</f>
+        <f aca="false">Hypothèses!G63</f>
         <v>30000000</v>
       </c>
       <c r="H53" s="15"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="13" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B54" s="6" t="s">
         <v>13</v>
@@ -4539,7 +4564,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="11" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B55" s="12"/>
       <c r="C55" s="12"/>
@@ -4580,7 +4605,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="6" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="B57" s="6" t="s">
         <v>20</v>
@@ -4609,7 +4634,7 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="6" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="B58" s="6" t="s">
         <v>13</v>
@@ -4635,12 +4660,12 @@
         <v>0</v>
       </c>
       <c r="H58" s="15" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="6" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="B59" s="6" t="s">
         <v>13</v>
@@ -4669,29 +4694,29 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="6" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B60" s="6" t="s">
         <v>13</v>
       </c>
       <c r="C60" s="25" t="n">
-        <f aca="false">MAX(0,C59)*Hypothèses!$C$63</f>
+        <f aca="false">MAX(0,C59)*Hypothèses!$C$64</f>
         <v>0</v>
       </c>
       <c r="D60" s="25" t="n">
-        <f aca="false">MAX(0,D59)*Hypothèses!$C$63</f>
+        <f aca="false">MAX(0,D59)*Hypothèses!$C$64</f>
         <v>0</v>
       </c>
       <c r="E60" s="25" t="n">
-        <f aca="false">MAX(0,E59)*Hypothèses!$C$63</f>
+        <f aca="false">MAX(0,E59)*Hypothèses!$C$64</f>
         <v>0</v>
       </c>
       <c r="F60" s="25" t="n">
-        <f aca="false">MAX(0,F59)*Hypothèses!$C$63</f>
+        <f aca="false">MAX(0,F59)*Hypothèses!$C$64</f>
         <v>0</v>
       </c>
       <c r="G60" s="25" t="n">
-        <f aca="false">MAX(0,G59)*Hypothèses!$C$63</f>
+        <f aca="false">MAX(0,G59)*Hypothèses!$C$64</f>
         <v>101653687.5</v>
       </c>
       <c r="H60" s="15"/>
@@ -4727,7 +4752,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="11" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="B62" s="12"/>
       <c r="C62" s="12"/>
@@ -4768,7 +4793,7 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="6" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="B64" s="6" t="s">
         <v>13</v>
@@ -4794,7 +4819,7 @@
         <v>304961062.5</v>
       </c>
       <c r="H64" s="15" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4828,10 +4853,10 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="6" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="C66" s="24" t="n">
         <f aca="false">IF(C56&gt;0,1,0)</f>
@@ -4857,7 +4882,7 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="11" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="12"/>
@@ -4898,7 +4923,7 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="6" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="B69" s="6" t="s">
         <v>25</v>
@@ -4927,7 +4952,7 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="6" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="B70" s="6" t="s">
         <v>25</v>
@@ -4956,64 +4981,64 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="6" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="B71" s="6" t="s">
         <v>25</v>
       </c>
       <c r="C71" s="24" t="n">
-        <f aca="false">IF(Hypothèses!C8=0,0,Hypothèses!C56/Hypothèses!C8)</f>
+        <f aca="false">IF(Hypothèses!C8=0,0,Hypothèses!C57/Hypothèses!C8)</f>
         <v>4285.71428571429</v>
       </c>
       <c r="D71" s="24" t="n">
-        <f aca="false">IF(Hypothèses!D8=0,0,Hypothèses!D56/Hypothèses!D8)</f>
+        <f aca="false">IF(Hypothèses!D8=0,0,Hypothèses!D57/Hypothèses!D8)</f>
         <v>3250</v>
       </c>
       <c r="E71" s="24" t="n">
-        <f aca="false">IF(Hypothèses!E8=0,0,Hypothèses!E56/Hypothèses!E8)</f>
+        <f aca="false">IF(Hypothèses!E8=0,0,Hypothèses!E57/Hypothèses!E8)</f>
         <v>2666.66666666667</v>
       </c>
       <c r="F71" s="24" t="n">
-        <f aca="false">IF(Hypothèses!F8=0,0,Hypothèses!F56/Hypothèses!F8)</f>
+        <f aca="false">IF(Hypothèses!F8=0,0,Hypothèses!F57/Hypothèses!F8)</f>
         <v>2291.66666666667</v>
       </c>
       <c r="G71" s="24" t="n">
-        <f aca="false">IF(Hypothèses!G8=0,0,Hypothèses!G56/Hypothèses!G8)</f>
+        <f aca="false">IF(Hypothèses!G8=0,0,Hypothèses!G57/Hypothèses!G8)</f>
         <v>2000</v>
       </c>
       <c r="H71" s="15" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="6" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="B72" s="6" t="s">
         <v>25</v>
       </c>
       <c r="C72" s="24" t="n">
-        <f aca="false">C70*Hypothèses!$C$64</f>
+        <f aca="false">C70*Hypothèses!$C$65</f>
         <v>-2467.97142857143</v>
       </c>
       <c r="D72" s="24" t="n">
-        <f aca="false">D70*Hypothèses!$C$64</f>
+        <f aca="false">D70*Hypothèses!$C$65</f>
         <v>3852.05706521739</v>
       </c>
       <c r="E72" s="24" t="n">
-        <f aca="false">E70*Hypothèses!$C$64</f>
+        <f aca="false">E70*Hypothèses!$C$65</f>
         <v>8199.07258064516</v>
       </c>
       <c r="F72" s="24" t="n">
-        <f aca="false">F70*Hypothèses!$C$64</f>
+        <f aca="false">F70*Hypothèses!$C$65</f>
         <v>11361.5612903226</v>
       </c>
       <c r="G72" s="24" t="n">
-        <f aca="false">G70*Hypothèses!$C$64</f>
+        <f aca="false">G70*Hypothèses!$C$65</f>
         <v>14522.2714285714</v>
       </c>
       <c r="H72" s="15" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5044,7 +5069,7 @@
         <v>7.26113571428571</v>
       </c>
       <c r="H73" s="15" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
     </row>
   </sheetData>
@@ -5072,7 +5097,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -5084,12 +5109,12 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="B4" s="29" t="n">
         <v>0.01</v>
@@ -5112,23 +5137,23 @@
         <v>0.005</v>
       </c>
       <c r="B5" s="25" t="n">
-        <f aca="false">Projections!$E$56+Projections!$E$14*(B$4-Hypothèses!$C$38)-Projections!$E$12*($A5-Hypothèses!$E$45)</f>
+        <f aca="false">Projections!$E$56+Projections!$E$14*(B$4-Hypothèses!$C$39)-Projections!$E$12*($A5-Hypothèses!$E$46)</f>
         <v>-255975687.5</v>
       </c>
       <c r="C5" s="25" t="n">
-        <f aca="false">Projections!$E$56+Projections!$E$14*(C$4-Hypothèses!$C$38)-Projections!$E$12*($A5-Hypothèses!$E$45)</f>
+        <f aca="false">Projections!$E$56+Projections!$E$14*(C$4-Hypothèses!$C$39)-Projections!$E$12*($A5-Hypothèses!$E$46)</f>
         <v>-234789125</v>
       </c>
       <c r="D5" s="25" t="n">
-        <f aca="false">Projections!$E$56+Projections!$E$14*(D$4-Hypothèses!$C$38)-Projections!$E$12*($A5-Hypothèses!$E$45)</f>
+        <f aca="false">Projections!$E$56+Projections!$E$14*(D$4-Hypothèses!$C$39)-Projections!$E$12*($A5-Hypothèses!$E$46)</f>
         <v>-213602562.5</v>
       </c>
       <c r="E5" s="25" t="n">
-        <f aca="false">Projections!$E$56+Projections!$E$14*(E$4-Hypothèses!$C$38)-Projections!$E$12*($A5-Hypothèses!$E$45)</f>
+        <f aca="false">Projections!$E$56+Projections!$E$14*(E$4-Hypothèses!$C$39)-Projections!$E$12*($A5-Hypothèses!$E$46)</f>
         <v>-192416000</v>
       </c>
       <c r="F5" s="25" t="n">
-        <f aca="false">Projections!$E$56+Projections!$E$14*(F$4-Hypothèses!$C$38)-Projections!$E$12*($A5-Hypothèses!$E$45)</f>
+        <f aca="false">Projections!$E$56+Projections!$E$14*(F$4-Hypothèses!$C$39)-Projections!$E$12*($A5-Hypothèses!$E$46)</f>
         <v>-171229437.5</v>
       </c>
     </row>
@@ -5137,23 +5162,23 @@
         <v>0.0065</v>
       </c>
       <c r="B6" s="25" t="n">
-        <f aca="false">Projections!$E$56+Projections!$E$14*(B$4-Hypothèses!$C$38)-Projections!$E$12*($A6-Hypothèses!$E$45)</f>
+        <f aca="false">Projections!$E$56+Projections!$E$14*(B$4-Hypothèses!$C$39)-Projections!$E$12*($A6-Hypothèses!$E$46)</f>
         <v>-287363187.5</v>
       </c>
       <c r="C6" s="25" t="n">
-        <f aca="false">Projections!$E$56+Projections!$E$14*(C$4-Hypothèses!$C$38)-Projections!$E$12*($A6-Hypothèses!$E$45)</f>
+        <f aca="false">Projections!$E$56+Projections!$E$14*(C$4-Hypothèses!$C$39)-Projections!$E$12*($A6-Hypothèses!$E$46)</f>
         <v>-266176625</v>
       </c>
       <c r="D6" s="25" t="n">
-        <f aca="false">Projections!$E$56+Projections!$E$14*(D$4-Hypothèses!$C$38)-Projections!$E$12*($A6-Hypothèses!$E$45)</f>
+        <f aca="false">Projections!$E$56+Projections!$E$14*(D$4-Hypothèses!$C$39)-Projections!$E$12*($A6-Hypothèses!$E$46)</f>
         <v>-244990062.5</v>
       </c>
       <c r="E6" s="25" t="n">
-        <f aca="false">Projections!$E$56+Projections!$E$14*(E$4-Hypothèses!$C$38)-Projections!$E$12*($A6-Hypothèses!$E$45)</f>
+        <f aca="false">Projections!$E$56+Projections!$E$14*(E$4-Hypothèses!$C$39)-Projections!$E$12*($A6-Hypothèses!$E$46)</f>
         <v>-223803500</v>
       </c>
       <c r="F6" s="25" t="n">
-        <f aca="false">Projections!$E$56+Projections!$E$14*(F$4-Hypothèses!$C$38)-Projections!$E$12*($A6-Hypothèses!$E$45)</f>
+        <f aca="false">Projections!$E$56+Projections!$E$14*(F$4-Hypothèses!$C$39)-Projections!$E$12*($A6-Hypothèses!$E$46)</f>
         <v>-202616937.5</v>
       </c>
     </row>
@@ -5162,23 +5187,23 @@
         <v>0.008</v>
       </c>
       <c r="B7" s="25" t="n">
-        <f aca="false">Projections!$E$56+Projections!$E$14*(B$4-Hypothèses!$C$38)-Projections!$E$12*($A7-Hypothèses!$E$45)</f>
+        <f aca="false">Projections!$E$56+Projections!$E$14*(B$4-Hypothèses!$C$39)-Projections!$E$12*($A7-Hypothèses!$E$46)</f>
         <v>-318750687.5</v>
       </c>
       <c r="C7" s="25" t="n">
-        <f aca="false">Projections!$E$56+Projections!$E$14*(C$4-Hypothèses!$C$38)-Projections!$E$12*($A7-Hypothèses!$E$45)</f>
+        <f aca="false">Projections!$E$56+Projections!$E$14*(C$4-Hypothèses!$C$39)-Projections!$E$12*($A7-Hypothèses!$E$46)</f>
         <v>-297564125</v>
       </c>
       <c r="D7" s="30" t="n">
-        <f aca="false">Projections!$E$56+Projections!$E$14*(D$4-Hypothèses!$C$38)-Projections!$E$12*($A7-Hypothèses!$E$45)</f>
+        <f aca="false">Projections!$E$56+Projections!$E$14*(D$4-Hypothèses!$C$39)-Projections!$E$12*($A7-Hypothèses!$E$46)</f>
         <v>-276377562.5</v>
       </c>
       <c r="E7" s="25" t="n">
-        <f aca="false">Projections!$E$56+Projections!$E$14*(E$4-Hypothèses!$C$38)-Projections!$E$12*($A7-Hypothèses!$E$45)</f>
+        <f aca="false">Projections!$E$56+Projections!$E$14*(E$4-Hypothèses!$C$39)-Projections!$E$12*($A7-Hypothèses!$E$46)</f>
         <v>-255191000</v>
       </c>
       <c r="F7" s="25" t="n">
-        <f aca="false">Projections!$E$56+Projections!$E$14*(F$4-Hypothèses!$C$38)-Projections!$E$12*($A7-Hypothèses!$E$45)</f>
+        <f aca="false">Projections!$E$56+Projections!$E$14*(F$4-Hypothèses!$C$39)-Projections!$E$12*($A7-Hypothèses!$E$46)</f>
         <v>-234004437.5</v>
       </c>
     </row>
@@ -5187,23 +5212,23 @@
         <v>0.01</v>
       </c>
       <c r="B8" s="25" t="n">
-        <f aca="false">Projections!$E$56+Projections!$E$14*(B$4-Hypothèses!$C$38)-Projections!$E$12*($A8-Hypothèses!$E$45)</f>
+        <f aca="false">Projections!$E$56+Projections!$E$14*(B$4-Hypothèses!$C$39)-Projections!$E$12*($A8-Hypothèses!$E$46)</f>
         <v>-360600687.5</v>
       </c>
       <c r="C8" s="25" t="n">
-        <f aca="false">Projections!$E$56+Projections!$E$14*(C$4-Hypothèses!$C$38)-Projections!$E$12*($A8-Hypothèses!$E$45)</f>
+        <f aca="false">Projections!$E$56+Projections!$E$14*(C$4-Hypothèses!$C$39)-Projections!$E$12*($A8-Hypothèses!$E$46)</f>
         <v>-339414125</v>
       </c>
       <c r="D8" s="25" t="n">
-        <f aca="false">Projections!$E$56+Projections!$E$14*(D$4-Hypothèses!$C$38)-Projections!$E$12*($A8-Hypothèses!$E$45)</f>
+        <f aca="false">Projections!$E$56+Projections!$E$14*(D$4-Hypothèses!$C$39)-Projections!$E$12*($A8-Hypothèses!$E$46)</f>
         <v>-318227562.5</v>
       </c>
       <c r="E8" s="25" t="n">
-        <f aca="false">Projections!$E$56+Projections!$E$14*(E$4-Hypothèses!$C$38)-Projections!$E$12*($A8-Hypothèses!$E$45)</f>
+        <f aca="false">Projections!$E$56+Projections!$E$14*(E$4-Hypothèses!$C$39)-Projections!$E$12*($A8-Hypothèses!$E$46)</f>
         <v>-297041000</v>
       </c>
       <c r="F8" s="25" t="n">
-        <f aca="false">Projections!$E$56+Projections!$E$14*(F$4-Hypothèses!$C$38)-Projections!$E$12*($A8-Hypothèses!$E$45)</f>
+        <f aca="false">Projections!$E$56+Projections!$E$14*(F$4-Hypothèses!$C$39)-Projections!$E$12*($A8-Hypothèses!$E$46)</f>
         <v>-275854437.5</v>
       </c>
     </row>
@@ -5212,29 +5237,29 @@
         <v>0.015</v>
       </c>
       <c r="B9" s="25" t="n">
-        <f aca="false">Projections!$E$56+Projections!$E$14*(B$4-Hypothèses!$C$38)-Projections!$E$12*($A9-Hypothèses!$E$45)</f>
+        <f aca="false">Projections!$E$56+Projections!$E$14*(B$4-Hypothèses!$C$39)-Projections!$E$12*($A9-Hypothèses!$E$46)</f>
         <v>-465225687.5</v>
       </c>
       <c r="C9" s="25" t="n">
-        <f aca="false">Projections!$E$56+Projections!$E$14*(C$4-Hypothèses!$C$38)-Projections!$E$12*($A9-Hypothèses!$E$45)</f>
+        <f aca="false">Projections!$E$56+Projections!$E$14*(C$4-Hypothèses!$C$39)-Projections!$E$12*($A9-Hypothèses!$E$46)</f>
         <v>-444039125</v>
       </c>
       <c r="D9" s="25" t="n">
-        <f aca="false">Projections!$E$56+Projections!$E$14*(D$4-Hypothèses!$C$38)-Projections!$E$12*($A9-Hypothèses!$E$45)</f>
+        <f aca="false">Projections!$E$56+Projections!$E$14*(D$4-Hypothèses!$C$39)-Projections!$E$12*($A9-Hypothèses!$E$46)</f>
         <v>-422852562.5</v>
       </c>
       <c r="E9" s="25" t="n">
-        <f aca="false">Projections!$E$56+Projections!$E$14*(E$4-Hypothèses!$C$38)-Projections!$E$12*($A9-Hypothèses!$E$45)</f>
+        <f aca="false">Projections!$E$56+Projections!$E$14*(E$4-Hypothèses!$C$39)-Projections!$E$12*($A9-Hypothèses!$E$46)</f>
         <v>-401666000</v>
       </c>
       <c r="F9" s="25" t="n">
-        <f aca="false">Projections!$E$56+Projections!$E$14*(F$4-Hypothèses!$C$38)-Projections!$E$12*($A9-Hypothèses!$E$45)</f>
+        <f aca="false">Projections!$E$56+Projections!$E$14*(F$4-Hypothèses!$C$39)-Projections!$E$12*($A9-Hypothèses!$E$46)</f>
         <v>-380479437.5</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="31" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
     </row>
   </sheetData>

</xml_diff>